<commit_message>
QA: actualizar Excel y docs de Cooper/Beneficios (IMAS-4356 + IMAS-4435)
Casos de Prueba.xlsx: +6 CP en Funcionalidades Pendientes (TS-06
Beneficios) - banner Cooper 3 segmentos + menu, verificado Desktop y
Mobile. Dashboard: 308 total, 228 automatizados (74%).

Automation Vetify.xlsx: +2 filas en el roadmap (QA-AUTO-093/094).
Dashboard: 88 escenarios.

docs/user-stories: IMAS-4356 cerrado con seccion de resolucion (causa
raiz real = policyId de la cuenta, no segmento/clCuenta). IMAS-4435
nuevo, con el contrato real completo (10 criterios de aceptacion)
cruzado contra lo automatizado.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Automation Vetify.xlsx
+++ b/documentation/Automation Vetify.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\ike\vetify-automation\automation\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ike\vetify-automation\automation\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{929DFDDE-F32E-4095-8CAA-1179C3EEE175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D41B8FEA-BD83-4820-998D-D9F3C411D1C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="416">
   <si>
     <t>ID</t>
   </si>
@@ -1263,6 +1263,30 @@
   </si>
   <si>
     <t>Mismo caso que la fila anterior: las 3 partes estan automatizadas por separado (Compra 50%, Carga de credencial 100%, Solicitar videollamada 100%) pero nunca encadenadas en un solo test end-to-end. Candidato natural a automatizar primero entre los 2 journeys nuevos, porque sus 3 partes ya estan en mejor estado individualmente.</t>
+  </si>
+  <si>
+    <t>QA-AUTO-093</t>
+  </si>
+  <si>
+    <t>Banner Cooper en Home</t>
+  </si>
+  <si>
+    <t>Validar que el banner de Cooper se muestra en Home para los 3 segmentos (Vetify B2C, OSDE Capitado, OSDE Adquirente).</t>
+  </si>
+  <si>
+    <t>IMAS-4356/IMAS-4435. tests/projects/vetify-webapp/navigation.spec.ts TS-05, 3 casos, verificado Desktop y Mobile (Android).</t>
+  </si>
+  <si>
+    <t>QA-AUTO-094</t>
+  </si>
+  <si>
+    <t>Menu Beneficios - segmentacion Cooper/Vetify PLUS</t>
+  </si>
+  <si>
+    <t>Validar que el menu lateral (seccion Beneficios) muestra Cooper y Vetify PLUS para B2C, y solo Cooper para OSDE Capitado.</t>
+  </si>
+  <si>
+    <t>IMAS-4356/IMAS-4435. TS-04 TC-01/02/03, verificado Desktop y Mobile. OSDE Adquirente no automatizado a proposito: la segmentacion real depende del policyId (producto real) de la cuenta, no del segmento -- ver docs/conocimiento-sistema.md.</t>
   </si>
 </sst>
 </file>
@@ -1590,7 +1614,7 @@
                   <c:v>0.17857142857142858</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.5</c:v>
+                  <c:v>0.66666666666666674</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -1797,7 +1821,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>30</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2195,7 +2219,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -5079,6 +5103,70 @@
       </c>
       <c r="K87" t="s">
         <v>407</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>408</v>
+      </c>
+      <c r="B88" t="s">
+        <v>280</v>
+      </c>
+      <c r="C88" t="s">
+        <v>45</v>
+      </c>
+      <c r="D88" t="s">
+        <v>409</v>
+      </c>
+      <c r="E88" t="s">
+        <v>410</v>
+      </c>
+      <c r="F88" t="s">
+        <v>15</v>
+      </c>
+      <c r="G88" t="s">
+        <v>16</v>
+      </c>
+      <c r="H88">
+        <v>1</v>
+      </c>
+      <c r="I88">
+        <v>100</v>
+      </c>
+      <c r="K88" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>412</v>
+      </c>
+      <c r="B89" t="s">
+        <v>280</v>
+      </c>
+      <c r="C89" t="s">
+        <v>45</v>
+      </c>
+      <c r="D89" t="s">
+        <v>413</v>
+      </c>
+      <c r="E89" t="s">
+        <v>414</v>
+      </c>
+      <c r="F89" t="s">
+        <v>15</v>
+      </c>
+      <c r="G89" t="s">
+        <v>16</v>
+      </c>
+      <c r="H89">
+        <v>1</v>
+      </c>
+      <c r="I89">
+        <v>100</v>
+      </c>
+      <c r="K89" t="s">
+        <v>415</v>
       </c>
     </row>
   </sheetData>
@@ -5224,19 +5312,19 @@
       <c r="A8" s="7"/>
       <c r="B8" s="20">
         <f>COUNTA('Roadmap QA Automation'!A2:A1998)</f>
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C8" s="18"/>
       <c r="D8" s="7"/>
       <c r="E8" s="21">
         <f>IFERROR(AVERAGE('Roadmap QA Automation'!I2:I1998)/100,0)</f>
-        <v>0.38953488372093026</v>
+        <v>0.40340909090909094</v>
       </c>
       <c r="F8" s="18"/>
       <c r="G8" s="7"/>
       <c r="H8" s="19">
         <f>COUNTIF('Roadmap QA Automation'!I2:I1998,100)</f>
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I8" s="18"/>
       <c r="J8" s="7"/>
@@ -5516,11 +5604,11 @@
       </c>
       <c r="C24" s="7">
         <f>COUNTIF('Roadmap QA Automation'!B:B,LEFT(B24,3)&amp;"*")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D24" s="11">
         <f>IFERROR(AVERAGEIF('Roadmap QA Automation'!B:B,LEFT(B24,3)&amp;"*",'Roadmap QA Automation'!I:I)/100,0)</f>
-        <v>0.5</v>
+        <v>0.66666666666666674</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
@@ -5734,7 +5822,7 @@
       </c>
       <c r="C36" s="7">
         <f>COUNTIF('Roadmap QA Automation'!I:I,100)</f>
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
@@ -5819,11 +5907,11 @@
       </c>
       <c r="C42" s="7">
         <f>COUNTIF('Roadmap QA Automation'!G:G,B42)</f>
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D42" s="11">
         <f>IFERROR(AVERAGEIF('Roadmap QA Automation'!G:G,B42,'Roadmap QA Automation'!I:I)/100,0)</f>
-        <v>0.37698412698412698</v>
+        <v>0.39615384615384613</v>
       </c>
       <c r="E42" s="7"/>
       <c r="F42" s="7"/>
@@ -6015,11 +6103,11 @@
       </c>
       <c r="C53" s="7">
         <f>COUNTIF('Roadmap QA Automation'!C:C,B53)</f>
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D53" s="11">
         <f>IFERROR(AVERAGEIF('Roadmap QA Automation'!C:C,B53,'Roadmap QA Automation'!I:I)/100,0)</f>
-        <v>0.38970588235294118</v>
+        <v>0.40714285714285714</v>
       </c>
       <c r="E53" s="7"/>
       <c r="F53" s="7"/>
@@ -6167,6 +6255,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="96ffd99d-26d2-4d99-98b0-05d0b9b7ac4e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="823bb257-b027-4d06-8b2f-053335b328b1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101009F842B2145328244B4B47741AC555AE2" ma:contentTypeVersion="11" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="783508ae003506b91aa2be35b4ebc887">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="96ffd99d-26d2-4d99-98b0-05d0b9b7ac4e" xmlns:ns3="823bb257-b027-4d06-8b2f-053335b328b1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4b965eb5b8ebcdb894d7355c785d1653" ns2:_="" ns3:_="">
     <xsd:import namespace="96ffd99d-26d2-4d99-98b0-05d0b9b7ac4e"/>
@@ -6361,27 +6469,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{347876AB-BDAE-4A3D-A9BF-1638E774D861}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="96ffd99d-26d2-4d99-98b0-05d0b9b7ac4e"/>
+    <ds:schemaRef ds:uri="823bb257-b027-4d06-8b2f-053335b328b1"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="96ffd99d-26d2-4d99-98b0-05d0b9b7ac4e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="823bb257-b027-4d06-8b2f-053335b328b1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{211C9EF2-99F3-47CC-A9EA-437B32406790}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A512D99-C2FC-42B8-8FDB-89CED4284B88}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6398,23 +6505,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{211C9EF2-99F3-47CC-A9EA-437B32406790}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{347876AB-BDAE-4A3D-A9BF-1638E774D861}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="96ffd99d-26d2-4d99-98b0-05d0b9b7ac4e"/>
-    <ds:schemaRef ds:uri="823bb257-b027-4d06-8b2f-053335b328b1"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>